<commit_message>
Clear test/demo content, restore reusable templates
Remove the placeholder exhibition, artworks, and text entry used to
validate the build pipeline, reset the artwork sheet to a header-only
row and CV.md to an empty template, and bring back the copyable
_양식 folders for 전시/텍스트/블로그 (작품 no longer needs one now
that it's driven by the spreadsheet). Also make empty collections
render a friendly placeholder instead of a blank list.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/작품/작품리스트.xlsx
+++ b/content/작품/작품리스트.xlsx
@@ -1,116 +1,55 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="122211"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
-  <si>
-    <t>제목(국문)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>제목(영문)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>제작연도</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>재료(국문)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>재료(영문)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>사이즈</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>테스트</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Test</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>캔버스 위에 아크릴릭</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Acrylic on canvas</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>100 x 100 cm</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>참조 코드</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>테스트2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Test2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1020 x 1020 cm</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
   <numFmts count="1">
-    <numFmt numFmtId="176" formatCode="000"/>
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="8"/>
-      <name val="맑은 고딕"/>
-      <family val="3"/>
-      <charset val="129"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -125,39 +64,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -199,7 +118,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -234,7 +153,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -301,20 +220,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -436,98 +351,80 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="22.375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="17.125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="20.25" style="2" customWidth="1"/>
-    <col min="4" max="4" width="22.25" style="2" customWidth="1"/>
-    <col min="5" max="5" width="19.75" style="2" customWidth="1"/>
-    <col min="6" max="6" width="23.375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="19.5" style="4" customWidth="1"/>
-    <col min="8" max="16384" width="9" style="2"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G1"/>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="2">
-        <v>2026</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="2">
-        <v>2025</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="4">
-        <v>2</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>제목(국문)</v>
+      </c>
+      <c r="B1" t="str">
+        <v>제목(영문)</v>
+      </c>
+      <c r="C1" t="str">
+        <v>제작연도</v>
+      </c>
+      <c r="D1" t="str">
+        <v>재료(국문)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>재료(영문)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>사이즈</v>
+      </c>
+      <c r="G1" t="str">
+        <v>참조 코드</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Restore demo content for showing the workflow
Reverting the earlier cleanup — this content is meant to stay as a
working example (exhibition, artworks, CV entries) so the intended
folder/file structure can be demonstrated hands-on.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/작품/작품리스트.xlsx
+++ b/content/작품/작품리스트.xlsx
@@ -1,55 +1,116 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <bookViews>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+  </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="122211"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
+  <si>
+    <t>제목(국문)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>제목(영문)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>제작연도</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>재료(국문)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>재료(영문)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>사이즈</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>테스트</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Test</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>캔버스 위에 아크릴릭</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Acrylic on canvas</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>100 x 100 cm</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>참조 코드</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>테스트2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Test2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1020 x 1020 cm</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="176" formatCode="000"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -64,19 +125,39 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -118,7 +199,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -153,7 +234,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -220,16 +301,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -351,80 +436,98 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22.375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="17.125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="20.25" style="2" customWidth="1"/>
+    <col min="4" max="4" width="22.25" style="2" customWidth="1"/>
+    <col min="5" max="5" width="19.75" style="2" customWidth="1"/>
+    <col min="6" max="6" width="23.375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="19.5" style="4" customWidth="1"/>
+    <col min="8" max="16384" width="9" style="2"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>제목(국문)</v>
-      </c>
-      <c r="B1" t="str">
-        <v>제목(영문)</v>
-      </c>
-      <c r="C1" t="str">
-        <v>제작연도</v>
-      </c>
-      <c r="D1" t="str">
-        <v>재료(국문)</v>
-      </c>
-      <c r="E1" t="str">
-        <v>재료(영문)</v>
-      </c>
-      <c r="F1" t="str">
-        <v>사이즈</v>
-      </c>
-      <c r="G1" t="str">
-        <v>참조 코드</v>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="4">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
-  </ignoredErrors>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>